<commit_message>
chore(bd): añade hojas simulacro_config (54 filas, 3 áreas) y simulacros al BD maestro
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BASE_DATOS_GUYTON.xlsx
+++ b/BASE_DATOS_GUYTON.xlsx
@@ -20,6 +20,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="materiales" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="asistencias" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="anuncios" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="simulacro_config" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="simulacros" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -939,7 +941,6 @@
           <t>presencial</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
           <t>programada</t>
@@ -1064,7 +1065,6 @@
           <t>https://drive.google.com/file/d/DEMO-practica-1/view</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>2026-07-13</t>
@@ -1170,7 +1170,6 @@
           <t>https://drive.google.com/file/d/DEMO-grabacion-1/view</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
           <t>2026-07-15</t>
@@ -1267,7 +1266,6 @@
           <t>usr-demo-3</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1373,7 +1371,6 @@
           <t>anu-demo-1</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>Bienvenida al ciclo 2026-II (DEMO)</t>
@@ -1444,6 +1441,1278 @@
       <c r="H3" t="inlineStr">
         <is>
           <t>publicado</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>curso</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>preguntas</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>puntos_pregunta</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>ponderacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Aritmética</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E2" t="n">
+        <v>5.201</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Álgebra</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E3" t="n">
+        <v>5.202</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Geometría</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E4" t="n">
+        <v>5.303</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Trigonometría</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="n">
+        <v>10</v>
+      </c>
+      <c r="E5" t="n">
+        <v>5.404</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E6" t="n">
+        <v>5.905</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Química</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E7" t="n">
+        <v>5.406</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Biología y Anatomía</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3.177</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Psicología y Filosofía</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" t="n">
+        <v>10</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3.802</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Geografía</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="n">
+        <v>10</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2.576</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Historia</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" t="n">
+        <v>10</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3.701</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Educación Cívica</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" t="n">
+        <v>10</v>
+      </c>
+      <c r="E12" t="n">
+        <v>3.101</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Economía</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" t="n">
+        <v>10</v>
+      </c>
+      <c r="E13" t="n">
+        <v>3.502</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Comunicación</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" t="n">
+        <v>10</v>
+      </c>
+      <c r="E14" t="n">
+        <v>3.352</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Literatura</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" t="n">
+        <v>10</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2.501</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Razonamiento Matemático</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>6</v>
+      </c>
+      <c r="D16" t="n">
+        <v>10</v>
+      </c>
+      <c r="E16" t="n">
+        <v>7.603</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Razonamiento Verbal</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>6</v>
+      </c>
+      <c r="D17" t="n">
+        <v>10</v>
+      </c>
+      <c r="E17" t="n">
+        <v>7.103</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" t="n">
+        <v>10</v>
+      </c>
+      <c r="E18" t="n">
+        <v>4.087</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Quechua y aimara</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="n">
+        <v>10</v>
+      </c>
+      <c r="E19" t="n">
+        <v>4.087</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Biomédicas</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Aritmética</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" t="n">
+        <v>10</v>
+      </c>
+      <c r="E20" t="n">
+        <v>3.331</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Biomédicas</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Álgebra</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" t="n">
+        <v>10</v>
+      </c>
+      <c r="E21" t="n">
+        <v>3.202</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Biomédicas</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Geometría</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>3</v>
+      </c>
+      <c r="D22" t="n">
+        <v>10</v>
+      </c>
+      <c r="E22" t="n">
+        <v>3.301</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Biomédicas</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Trigonometría</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" t="n">
+        <v>10</v>
+      </c>
+      <c r="E23" t="n">
+        <v>3.404</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Biomédicas</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" t="n">
+        <v>10</v>
+      </c>
+      <c r="E24" t="n">
+        <v>5.505</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Biomédicas</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Química</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>5</v>
+      </c>
+      <c r="D25" t="n">
+        <v>10</v>
+      </c>
+      <c r="E25" t="n">
+        <v>6.623</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Biomédicas</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Biología y Anatomía</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>6</v>
+      </c>
+      <c r="D26" t="n">
+        <v>10</v>
+      </c>
+      <c r="E26" t="n">
+        <v>7.816</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Biomédicas</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Psicología y Filosofía</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>4</v>
+      </c>
+      <c r="D27" t="n">
+        <v>10</v>
+      </c>
+      <c r="E27" t="n">
+        <v>4.006</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Biomédicas</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Geografía</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" t="n">
+        <v>10</v>
+      </c>
+      <c r="E28" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Biomédicas</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Historia</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>2</v>
+      </c>
+      <c r="D29" t="n">
+        <v>10</v>
+      </c>
+      <c r="E29" t="n">
+        <v>3.302</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Biomédicas</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Educación Cívica</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>2</v>
+      </c>
+      <c r="D30" t="n">
+        <v>10</v>
+      </c>
+      <c r="E30" t="n">
+        <v>3.571</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Biomédicas</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Economía</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>2</v>
+      </c>
+      <c r="D31" t="n">
+        <v>10</v>
+      </c>
+      <c r="E31" t="n">
+        <v>3.406</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Biomédicas</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Comunicación</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D32" t="n">
+        <v>10</v>
+      </c>
+      <c r="E32" t="n">
+        <v>3.302</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Biomédicas</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Literatura</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>2</v>
+      </c>
+      <c r="D33" t="n">
+        <v>10</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2.805</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Biomédicas</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Razonamiento Matemático</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>6</v>
+      </c>
+      <c r="D34" t="n">
+        <v>10</v>
+      </c>
+      <c r="E34" t="n">
+        <v>7.201</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Biomédicas</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Razonamiento Verbal</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>6</v>
+      </c>
+      <c r="D35" t="n">
+        <v>10</v>
+      </c>
+      <c r="E35" t="n">
+        <v>7.201</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Biomédicas</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" t="n">
+        <v>10</v>
+      </c>
+      <c r="E36" t="n">
+        <v>4.087</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Biomédicas</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Quechua y aimara</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" t="n">
+        <v>10</v>
+      </c>
+      <c r="E37" t="n">
+        <v>4.087</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Sociales</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Aritmética</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" t="n">
+        <v>10</v>
+      </c>
+      <c r="E38" t="n">
+        <v>3.331</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Sociales</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Álgebra</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>3</v>
+      </c>
+      <c r="D39" t="n">
+        <v>10</v>
+      </c>
+      <c r="E39" t="n">
+        <v>3.185</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Sociales</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Geometría</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>2</v>
+      </c>
+      <c r="D40" t="n">
+        <v>10</v>
+      </c>
+      <c r="E40" t="n">
+        <v>3.12</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Sociales</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Trigonometría</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>2</v>
+      </c>
+      <c r="D41" t="n">
+        <v>10</v>
+      </c>
+      <c r="E41" t="n">
+        <v>3.12</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Sociales</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>2</v>
+      </c>
+      <c r="D42" t="n">
+        <v>10</v>
+      </c>
+      <c r="E42" t="n">
+        <v>2.302</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Sociales</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Química</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>2</v>
+      </c>
+      <c r="D43" t="n">
+        <v>10</v>
+      </c>
+      <c r="E43" t="n">
+        <v>2.404</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Sociales</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Biología y Anatomía</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>2</v>
+      </c>
+      <c r="D44" t="n">
+        <v>10</v>
+      </c>
+      <c r="E44" t="n">
+        <v>2.504</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Sociales</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Psicología y Filosofía</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>4</v>
+      </c>
+      <c r="D45" t="n">
+        <v>10</v>
+      </c>
+      <c r="E45" t="n">
+        <v>4.807</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Sociales</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Geografía</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>4</v>
+      </c>
+      <c r="D46" t="n">
+        <v>10</v>
+      </c>
+      <c r="E46" t="n">
+        <v>4.907</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Sociales</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Historia</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>4</v>
+      </c>
+      <c r="D47" t="n">
+        <v>10</v>
+      </c>
+      <c r="E47" t="n">
+        <v>5.805</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Sociales</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Educación Cívica</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>4</v>
+      </c>
+      <c r="D48" t="n">
+        <v>10</v>
+      </c>
+      <c r="E48" t="n">
+        <v>6.576</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Sociales</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Economía</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>4</v>
+      </c>
+      <c r="D49" t="n">
+        <v>10</v>
+      </c>
+      <c r="E49" t="n">
+        <v>4.607</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Sociales</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Comunicación</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D50" t="n">
+        <v>10</v>
+      </c>
+      <c r="E50" t="n">
+        <v>6.09</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Sociales</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Literatura</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>4</v>
+      </c>
+      <c r="D51" t="n">
+        <v>10</v>
+      </c>
+      <c r="E51" t="n">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Sociales</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Razonamiento Matemático</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>6</v>
+      </c>
+      <c r="D52" t="n">
+        <v>10</v>
+      </c>
+      <c r="E52" t="n">
+        <v>7.203</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Sociales</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Razonamiento Verbal</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>6</v>
+      </c>
+      <c r="D53" t="n">
+        <v>10</v>
+      </c>
+      <c r="E53" t="n">
+        <v>7.603</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Sociales</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>2</v>
+      </c>
+      <c r="D54" t="n">
+        <v>10</v>
+      </c>
+      <c r="E54" t="n">
+        <v>4.087</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Sociales</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Quechua y aimara</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" t="n">
+        <v>10</v>
+      </c>
+      <c r="E55" t="n">
+        <v>4.087</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>id_simulacro</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>id_usuario</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>dni</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>nombre</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>fecha</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>puntaje_max</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>correctas</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>porcentaje</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>detalle</t>
         </is>
       </c>
     </row>
@@ -1523,7 +2792,6 @@
           <t>drive_root_id</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>ID de la carpeta raiz de Google Drive (vacio hasta que el usuario la comparta)</t>
@@ -1706,7 +2974,6 @@
           <t>1111</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>activo</t>
@@ -1759,7 +3026,6 @@
           <t>2222</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>activo</t>
@@ -1812,7 +3078,6 @@
           <t>3333</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>activo</t>
@@ -1865,7 +3130,6 @@
           <t>4444</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>activo</t>
@@ -1918,7 +3182,6 @@
           <t>5555</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>activo</t>
@@ -2292,7 +3555,6 @@
           <t>cur-demo-1</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
         <v>1</v>
       </c>
@@ -2583,7 +3845,6 @@
           <t>2026-07-18</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>plin</t>
@@ -2599,7 +3860,6 @@
           <t>PLIN-000456</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">

</xml_diff>

<commit_message>
chore(bd): columna clave en simulacro_config del BD maestro
</commit_message>
<xml_diff>
--- a/BASE_DATOS_GUYTON.xlsx
+++ b/BASE_DATOS_GUYTON.xlsx
@@ -1455,7 +1455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1463,6 +1463,7 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1491,6 +1492,11 @@
           <t>ponderacion</t>
         </is>
       </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>clave</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1512,6 +1518,7 @@
       <c r="E2" t="n">
         <v>5.201</v>
       </c>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1533,6 +1540,7 @@
       <c r="E3" t="n">
         <v>5.202</v>
       </c>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1554,6 +1562,7 @@
       <c r="E4" t="n">
         <v>5.303</v>
       </c>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1575,6 +1584,7 @@
       <c r="E5" t="n">
         <v>5.404</v>
       </c>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1596,6 +1606,7 @@
       <c r="E6" t="n">
         <v>5.905</v>
       </c>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1617,6 +1628,7 @@
       <c r="E7" t="n">
         <v>5.406</v>
       </c>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1638,6 +1650,7 @@
       <c r="E8" t="n">
         <v>3.177</v>
       </c>
+      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1659,6 +1672,7 @@
       <c r="E9" t="n">
         <v>3.802</v>
       </c>
+      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1680,6 +1694,7 @@
       <c r="E10" t="n">
         <v>2.576</v>
       </c>
+      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1701,6 +1716,7 @@
       <c r="E11" t="n">
         <v>3.701</v>
       </c>
+      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1722,6 +1738,7 @@
       <c r="E12" t="n">
         <v>3.101</v>
       </c>
+      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1743,6 +1760,7 @@
       <c r="E13" t="n">
         <v>3.502</v>
       </c>
+      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1764,6 +1782,7 @@
       <c r="E14" t="n">
         <v>3.352</v>
       </c>
+      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1785,6 +1804,7 @@
       <c r="E15" t="n">
         <v>2.501</v>
       </c>
+      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1806,6 +1826,7 @@
       <c r="E16" t="n">
         <v>7.603</v>
       </c>
+      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1827,6 +1848,7 @@
       <c r="E17" t="n">
         <v>7.103</v>
       </c>
+      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1848,6 +1870,7 @@
       <c r="E18" t="n">
         <v>4.087</v>
       </c>
+      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1869,6 +1892,7 @@
       <c r="E19" t="n">
         <v>4.087</v>
       </c>
+      <c r="F19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1890,6 +1914,7 @@
       <c r="E20" t="n">
         <v>3.331</v>
       </c>
+      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1911,6 +1936,7 @@
       <c r="E21" t="n">
         <v>3.202</v>
       </c>
+      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1932,6 +1958,7 @@
       <c r="E22" t="n">
         <v>3.301</v>
       </c>
+      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1953,6 +1980,7 @@
       <c r="E23" t="n">
         <v>3.404</v>
       </c>
+      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1974,6 +2002,7 @@
       <c r="E24" t="n">
         <v>5.505</v>
       </c>
+      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1995,6 +2024,7 @@
       <c r="E25" t="n">
         <v>6.623</v>
       </c>
+      <c r="F25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2016,6 +2046,7 @@
       <c r="E26" t="n">
         <v>7.816</v>
       </c>
+      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2037,6 +2068,7 @@
       <c r="E27" t="n">
         <v>4.006</v>
       </c>
+      <c r="F27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2058,6 +2090,7 @@
       <c r="E28" t="n">
         <v>2.8</v>
       </c>
+      <c r="F28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2079,6 +2112,7 @@
       <c r="E29" t="n">
         <v>3.302</v>
       </c>
+      <c r="F29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2100,6 +2134,7 @@
       <c r="E30" t="n">
         <v>3.571</v>
       </c>
+      <c r="F30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2121,6 +2156,7 @@
       <c r="E31" t="n">
         <v>3.406</v>
       </c>
+      <c r="F31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2142,6 +2178,7 @@
       <c r="E32" t="n">
         <v>3.302</v>
       </c>
+      <c r="F32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2163,6 +2200,7 @@
       <c r="E33" t="n">
         <v>2.805</v>
       </c>
+      <c r="F33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2184,6 +2222,7 @@
       <c r="E34" t="n">
         <v>7.201</v>
       </c>
+      <c r="F34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2205,6 +2244,7 @@
       <c r="E35" t="n">
         <v>7.201</v>
       </c>
+      <c r="F35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2226,6 +2266,7 @@
       <c r="E36" t="n">
         <v>4.087</v>
       </c>
+      <c r="F36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2247,6 +2288,7 @@
       <c r="E37" t="n">
         <v>4.087</v>
       </c>
+      <c r="F37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2268,6 +2310,7 @@
       <c r="E38" t="n">
         <v>3.331</v>
       </c>
+      <c r="F38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2289,6 +2332,7 @@
       <c r="E39" t="n">
         <v>3.185</v>
       </c>
+      <c r="F39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2310,6 +2354,7 @@
       <c r="E40" t="n">
         <v>3.12</v>
       </c>
+      <c r="F40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2331,6 +2376,7 @@
       <c r="E41" t="n">
         <v>3.12</v>
       </c>
+      <c r="F41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2352,6 +2398,7 @@
       <c r="E42" t="n">
         <v>2.302</v>
       </c>
+      <c r="F42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2373,6 +2420,7 @@
       <c r="E43" t="n">
         <v>2.404</v>
       </c>
+      <c r="F43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2394,6 +2442,7 @@
       <c r="E44" t="n">
         <v>2.504</v>
       </c>
+      <c r="F44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2415,6 +2464,7 @@
       <c r="E45" t="n">
         <v>4.807</v>
       </c>
+      <c r="F45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2436,6 +2486,7 @@
       <c r="E46" t="n">
         <v>4.907</v>
       </c>
+      <c r="F46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2457,6 +2508,7 @@
       <c r="E47" t="n">
         <v>5.805</v>
       </c>
+      <c r="F47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2478,6 +2530,7 @@
       <c r="E48" t="n">
         <v>6.576</v>
       </c>
+      <c r="F48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2499,6 +2552,7 @@
       <c r="E49" t="n">
         <v>4.607</v>
       </c>
+      <c r="F49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2520,6 +2574,7 @@
       <c r="E50" t="n">
         <v>6.09</v>
       </c>
+      <c r="F50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2541,6 +2596,7 @@
       <c r="E51" t="n">
         <v>4.3</v>
       </c>
+      <c r="F51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2562,6 +2618,7 @@
       <c r="E52" t="n">
         <v>7.203</v>
       </c>
+      <c r="F52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2583,6 +2640,7 @@
       <c r="E53" t="n">
         <v>7.603</v>
       </c>
+      <c r="F53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2604,6 +2662,7 @@
       <c r="E54" t="n">
         <v>4.087</v>
       </c>
+      <c r="F54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2625,6 +2684,7 @@
       <c r="E55" t="n">
         <v>4.087</v>
       </c>
+      <c r="F55" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>